<commit_message>
docs(ao): refresh v009 (EN+RU) — G85 hover comment corrected
Director correction 2026-05-05: hover comment rewritten to drop the
wrong attribution (DV UBS Swiss bridge / Armenia top-up) and instead
state the Brisen-side fact: EUR 2.5M arrived at LCG on 28 Apr 2026,
transmitted onward to RG7. Confirmed by Constantinos 27-28 Apr.

Aligned with baker-vault commit b4eefe4 + corrected dossier
curated/2026-05-04-ao-capital-call-7m-walkthrough.md.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs-site/ao/009_MOVIE_AO_Financing_Final_Reported_20260413.xlsx
+++ b/docs-site/ao/009_MOVIE_AO_Financing_Final_Reported_20260413.xlsx
@@ -5953,12 +5953,12 @@
   <commentList>
     <comment ref="G85" authorId="0" shapeId="0">
       <text>
-        <t>PAID — AO April DR#1 fulfilled.
-Settlement 24-27 Apr 2026 (mixed-source):
-  • USD 700K bridged from DV UBS Swiss private (Fri 24 Apr 2026)
-  • USD 1.8M from AO's Armenia account (27 Apr 2026)
-Eli→LCG payment orders executed 28 Apr 2026.
-Field-validated AO Baden-Baden 2026-05-04.
+        <t>PAID — AO April capital call DR#1 fulfilled.
+EUR 2.5M arrived at LCG on 28 April 2026 and was transmitted onward to RG7.
+Confirmed by Constantinos:
+  • 27 Apr 18:27: payment orders Eli→LCG filed for execution next day.
+  • 28 Apr 10:14: 'All the money's been moved today and is now in the right spots.'
+Field-validated AO Baden-Baden 2026-05-04. Director ratified 2026-05-05.
 See curated/2026-05-04-ao-capital-call-7m-walkthrough.md.</t>
       </text>
     </comment>

</xml_diff>